<commit_message>
Update data pipeline (auto)
</commit_message>
<xml_diff>
--- a/data/indicadores.xlsx
+++ b/data/indicadores.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +425,642 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Setor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cotacao</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Min_52_sem</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Max_52_sem</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Valor_de_mercado</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Nro_Acoes</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Patrim_Liq</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Receita_Liquida_12m</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Receita_Liquida_3m</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Lucro_Liquido_12m</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Lucro_Liquido_3m</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>P/L</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>DY</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>P/VP</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>ROE</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>LPA</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>VPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ABEV3</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bebidas</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="D2" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="E2" t="n">
+        <v>16.95</v>
+      </c>
+      <c r="F2" t="n">
+        <v>259155000000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>15763700000</v>
+      </c>
+      <c r="H2" t="n">
+        <v>90125800000</v>
+      </c>
+      <c r="I2" t="n">
+        <v>88209600000</v>
+      </c>
+      <c r="J2" t="n">
+        <v>22464500000</v>
+      </c>
+      <c r="K2" t="n">
+        <v>15577700000</v>
+      </c>
+      <c r="L2" t="n">
+        <v>3768260000</v>
+      </c>
+      <c r="M2" t="n">
+        <v>16.64</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.0522</v>
+      </c>
+      <c r="O2" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.1728</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="R2" t="n">
+        <v>5.72</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B3SA3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Serviços Financeiros Diversos</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>15.04</v>
+      </c>
+      <c r="D3" t="n">
+        <v>11.86</v>
+      </c>
+      <c r="E3" t="n">
+        <v>19.84</v>
+      </c>
+      <c r="F3" t="n">
+        <v>75899400000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5046500000</v>
+      </c>
+      <c r="H3" t="n">
+        <v>18255700000</v>
+      </c>
+      <c r="I3" t="n">
+        <v>11666100000</v>
+      </c>
+      <c r="J3" t="n">
+        <v>3201740000</v>
+      </c>
+      <c r="K3" t="n">
+        <v>4956510000</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1476970000</v>
+      </c>
+      <c r="M3" t="n">
+        <v>15.31</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.0418</v>
+      </c>
+      <c r="O3" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.2715</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="R3" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GGBR4</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Siderurgia e Metalurgia</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>23.29</v>
+      </c>
+      <c r="D4" t="n">
+        <v>15.31</v>
+      </c>
+      <c r="E4" t="n">
+        <v>24.65</v>
+      </c>
+      <c r="F4" t="n">
+        <v>46234300000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1985160000</v>
+      </c>
+      <c r="H4" t="n">
+        <v>52772500000</v>
+      </c>
+      <c r="I4" t="n">
+        <v>69198800000</v>
+      </c>
+      <c r="J4" t="n">
+        <v>16715700000</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1639580000</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1002050000</v>
+      </c>
+      <c r="M4" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.0295</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.0311</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="R4" t="n">
+        <v>26.58</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ITSA4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Intermediários Financeiros</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="D5" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>14.98</v>
+      </c>
+      <c r="F5" t="n">
+        <v>144208000000</v>
+      </c>
+      <c r="G5" t="n">
+        <v>11213700000</v>
+      </c>
+      <c r="H5" t="n">
+        <v>90196000000</v>
+      </c>
+      <c r="I5" t="n">
+        <v>8365000000</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2019000000</v>
+      </c>
+      <c r="K5" t="n">
+        <v>16983000000</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4410000000</v>
+      </c>
+      <c r="M5" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.0955</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.1883</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="R5" t="n">
+        <v>8.039999999999999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Petróleo, Gás e Biocombustíveis</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>38.54</v>
+      </c>
+      <c r="D6" t="n">
+        <v>27.94</v>
+      </c>
+      <c r="E6" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="F6" t="n">
+        <v>496732000000</v>
+      </c>
+      <c r="G6" t="n">
+        <v>12888700000</v>
+      </c>
+      <c r="H6" t="n">
+        <v>445189000000</v>
+      </c>
+      <c r="I6" t="n">
+        <v>498091000000</v>
+      </c>
+      <c r="J6" t="n">
+        <v>123686000000</v>
+      </c>
+      <c r="K6" t="n">
+        <v>107583000000</v>
+      </c>
+      <c r="L6" t="n">
+        <v>32663000000</v>
+      </c>
+      <c r="M6" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="O6" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.2417</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="R6" t="n">
+        <v>34.54</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RENT3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Diversos</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>40.96</v>
+      </c>
+      <c r="D7" t="n">
+        <v>30.54</v>
+      </c>
+      <c r="E7" t="n">
+        <v>52.33</v>
+      </c>
+      <c r="F7" t="n">
+        <v>46049600000</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1124260000</v>
+      </c>
+      <c r="H7" t="n">
+        <v>26309600000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>43926700000</v>
+      </c>
+      <c r="J7" t="n">
+        <v>12284400000</v>
+      </c>
+      <c r="K7" t="n">
+        <v>2254120000</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1221900000</v>
+      </c>
+      <c r="M7" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.0489</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.0857</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R7" t="n">
+        <v>23.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Madeira e Papel</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>42.93</v>
+      </c>
+      <c r="D8" t="n">
+        <v>40.43</v>
+      </c>
+      <c r="E8" t="n">
+        <v>58.98</v>
+      </c>
+      <c r="F8" t="n">
+        <v>54268600000</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1264120000</v>
+      </c>
+      <c r="H8" t="n">
+        <v>48036000000</v>
+      </c>
+      <c r="I8" t="n">
+        <v>49531200000</v>
+      </c>
+      <c r="J8" t="n">
+        <v>10968400000</v>
+      </c>
+      <c r="K8" t="n">
+        <v>11372800000</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4305400000</v>
+      </c>
+      <c r="M8" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="O8" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.2368</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>9</v>
+      </c>
+      <c r="R8" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VALE3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mineração</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>81.44</v>
+      </c>
+      <c r="D9" t="n">
+        <v>46.22</v>
+      </c>
+      <c r="E9" t="n">
+        <v>90.09</v>
+      </c>
+      <c r="F9" t="n">
+        <v>361525000000</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4439160000</v>
+      </c>
+      <c r="H9" t="n">
+        <v>191216000000</v>
+      </c>
+      <c r="I9" t="n">
+        <v>214864000000</v>
+      </c>
+      <c r="J9" t="n">
+        <v>48680000000</v>
+      </c>
+      <c r="K9" t="n">
+        <v>15603000000</v>
+      </c>
+      <c r="L9" t="n">
+        <v>9953000000</v>
+      </c>
+      <c r="M9" t="n">
+        <v>23.17</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.0688</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.08160000000000001</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="R9" t="n">
+        <v>43.07</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WEGE3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Máquinas e Equipamentos</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>42.83</v>
+      </c>
+      <c r="D10" t="n">
+        <v>34.22</v>
+      </c>
+      <c r="E10" t="n">
+        <v>53.93</v>
+      </c>
+      <c r="F10" t="n">
+        <v>179771000000</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4197320000</v>
+      </c>
+      <c r="H10" t="n">
+        <v>17746100000</v>
+      </c>
+      <c r="I10" t="n">
+        <v>40193900000</v>
+      </c>
+      <c r="J10" t="n">
+        <v>9468310000</v>
+      </c>
+      <c r="K10" t="n">
+        <v>6287370000</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1457190000</v>
+      </c>
+      <c r="M10" t="n">
+        <v>28.59</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.0506</v>
+      </c>
+      <c r="O10" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.3543</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.23</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>